<commit_message>
Version 1.0.0 Final before any change 12 May 2026
</commit_message>
<xml_diff>
--- a/SRC/Controller/HVAC_controller/State_Reward_action defintion.xlsx
+++ b/SRC/Controller/HVAC_controller/State_Reward_action defintion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YajuR\Desktop\Autonomy\Dwelling_simulator\SRC\Controller\HVAC_controller\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0DA101E-25AF-4F1F-BF2A-34CFB0EB7CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907F1F1E-8D06-4C62-B89E-5B4A1149B438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2F0CEAD1-91A2-44EE-9519-226D71FD8C97}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="14880" firstSheet="2" activeTab="2" xr2:uid="{2F0CEAD1-91A2-44EE-9519-226D71FD8C97}"/>
   </bookViews>
   <sheets>
     <sheet name="Reward" sheetId="1" r:id="rId1"/>
@@ -5304,6 +5304,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="696624863"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -13916,7 +13917,7 @@
         <v>30</v>
       </c>
       <c r="B39">
-        <f t="shared" si="4"/>
+        <f>(A39-AVERAGE(C$1:C$2))/$C$4</f>
         <v>2.5</v>
       </c>
       <c r="C39">

</xml_diff>